<commit_message>
🤖 [Robot Magazzino] Sincronizzazione database giacenza_schede.xlsx
</commit_message>
<xml_diff>
--- a/giacenza_schede.xlsx
+++ b/giacenza_schede.xlsx
@@ -1636,7 +1636,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>WINGAMING SRL</t>
+          <t>WINGAMING SRL - DEPOSITO AWP ASSEGNATE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1729,7 +1729,11 @@
         </is>
       </c>
       <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">

</xml_diff>